<commit_message>
feat: terminologia Asignatura+Grupo, soporte multi-cohorte (ISO 21001)
</commit_message>
<xml_diff>
--- a/uploads/FIS301 - Fisica Cuantica Aplicada-REV/bases_de_datos/CONTROL_VERSIONES_DOCUMENTAL.xlsx
+++ b/uploads/FIS301 - Fisica Cuantica Aplicada-REV/bases_de_datos/CONTROL_VERSIONES_DOCUMENTAL.xlsx
@@ -525,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -556,7 +556,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Registro Oficial de Versiones Vigentes y Trazabilidad de Evidencias Curriculares • Emisión: 06/09/2026 20:51</t>
+          <t>Registro Oficial de Versiones Vigentes y Trazabilidad de Evidencias Curriculares • Emisión: 06/09/2026 21:12</t>
         </is>
       </c>
     </row>
@@ -610,17 +610,17 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>DOC-CP2-BASE-FIS301Fi</t>
+          <t>DOC-CP2-VER-FIS301</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>BASE_INTEGRADA.xlsx</t>
+          <t>Libro Oficial de Control de Versiones y Trazabilidad Curricular</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>Datos Curriculares y Analíticos</t>
+          <t>Registro Maestro de Control de Versiones</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -630,22 +630,22 @@
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>06/09/2026 20:51</t>
+          <t>06/09/2026 21:12</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>Agente Etapa 1 - Preparador</t>
+          <t>Sistema de Gestión de Calidad (ISO 21001)</t>
         </is>
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Pipeline IA Autónomo</t>
+          <t>Edición Manual Docente</t>
         </is>
       </c>
       <c r="H6" s="10" t="inlineStr">
         <is>
-          <t>4c9a23391394b691...</t>
+          <t>82524f2d0f91b5aa...</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
@@ -657,17 +657,17 @@
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>DOC-CP2-VER-FIS301Fi</t>
+          <t>DOC-CP2-BASE-FIS301</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>CONTROL_VERSIONES_DOCUMENTAL.xlsx</t>
+          <t>Base de Datos Integrada y Curada</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Registro Oficial de Control Documental</t>
+          <t>Base de Datos de Aula Consolidada</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
@@ -677,22 +677,22 @@
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>06/09/2026 20:51</t>
+          <t>06/09/2026 21:12</t>
         </is>
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>Sistema de Gestión de Calidad</t>
+          <t>Agente Etapa 1 (Ingesta &amp; Fusión)</t>
         </is>
       </c>
       <c r="G7" s="11" t="inlineStr">
         <is>
-          <t>Edición Manual Docente</t>
+          <t>Pipeline IA Autónomo</t>
         </is>
       </c>
       <c r="H7" s="10" t="inlineStr">
         <is>
-          <t>e2565cec6a82578c...</t>
+          <t>4c9a23391394b691...</t>
         </is>
       </c>
       <c r="I7" s="11" t="inlineStr">
@@ -724,7 +724,7 @@
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>06/09/2026 20:52</t>
+          <t>06/09/2026 21:12</t>
         </is>
       </c>
       <c r="F8" s="10" t="inlineStr">
@@ -739,7 +739,7 @@
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
-          <t>522570a273052e62...</t>
+          <t>ed4bd53240327091...</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr">
@@ -751,17 +751,17 @@
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>DOC-DIR-CP2-INF3-FIS301</t>
+          <t>DOC-DIR-CP2-DUA-FIS301Fi</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Informe Analítico de Aprendizaje IA - FIS301 - Fisica Cuantica Aplicada</t>
+          <t>MATRIZ_ADAPTACIONES_DUA_FIS301_-_Fisica_Cuantica_Aplicada.docx</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>Informe Analítico Multidimensional</t>
+          <t>Matriz de Ajustes Razonables (Inclusión DUA)</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
@@ -771,25 +771,72 @@
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>06/09/2026 20:59</t>
+          <t>06/09/2026 21:12</t>
         </is>
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
-          <t>Agente Etapa 3 (Analítica &amp; Gemini IA)</t>
+          <t>Servicio DUA Institucional</t>
         </is>
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
-          <t>Pipeline IA Autónomo</t>
+          <t>Edición Manual Docente</t>
         </is>
       </c>
       <c r="H9" s="10" t="inlineStr">
         <is>
-          <t>138069782a4ef79d...</t>
+          <t>8d61021cfa5ad087...</t>
         </is>
       </c>
       <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>Aprobado Institucional</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>DOC-DIR-CP2-PDC-FIS301</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Plan de Aprendizaje Modular CBL - FIS301 - Fisica Cuantica Aplicada</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Planificación Didáctica Modular</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>06/09/2026 21:12</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>Motor de Planificación CBL / UbD</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>Edición Manual Docente</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>21c12f9558760d00...</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="inlineStr">
         <is>
           <t>Aprobado Institucional</t>
         </is>
@@ -811,7 +858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -882,12 +929,12 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>06/09/2026 20:51</t>
+          <t>06/09/2026 21:12</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>BASE_INTEGRADA.xlsx</t>
+          <t>Libro Oficial de Control de Versiones y Trazabilidad Curricular</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
@@ -897,17 +944,17 @@
       </c>
       <c r="E5" s="10" t="inlineStr">
         <is>
-          <t>Agente Etapa 1 - Preparador</t>
+          <t>Sistema de Gestión de Calidad (ISO 21001)</t>
         </is>
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>Consolidación inicial de 4 archivos crudos para 12 estudiantes.</t>
+          <t>Inicialización de la matriz de versiones y bitácora inmutable de auditoría.</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
-          <t>Aseguramiento de trazabilidad y limpieza de datos según norma ISO 21001.</t>
+          <t>Aseguramiento de la información documentada (ISO 21001:2018 Cláusula 7.5).</t>
         </is>
       </c>
     </row>
@@ -919,12 +966,12 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>06/09/2026 20:51</t>
+          <t>06/09/2026 21:12</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>CONTROL_VERSIONES_DOCUMENTAL.xlsx</t>
+          <t>Base de Datos Integrada y Curada</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -934,17 +981,17 @@
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>Sistema de Gestión de Calidad</t>
+          <t>Agente Etapa 1 (Ingesta &amp; Fusión)</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>Apertura de la bitácora inmutable y matriz de versiones de la asignatura.</t>
+          <t>Consolidación de planillas de asistencia, notas y evidencias en libro maestro.</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>Cumplimiento formal de la Cláusula 7.5 de ISO 21001 (Información Documentada).</t>
+          <t>Estandarización de datos de rendimiento académico para analítica de aprendizaje.</t>
         </is>
       </c>
     </row>
@@ -956,7 +1003,7 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>06/09/2026 20:52</t>
+          <t>06/09/2026 21:12</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
@@ -993,12 +1040,12 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>06/09/2026 20:59</t>
+          <t>06/09/2026 21:12</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>Informe Analítico de Aprendizaje IA - FIS301 - Fisica Cuantica Aplicada</t>
+          <t>MATRIZ_ADAPTACIONES_DUA_FIS301_-_Fisica_Cuantica_Aplicada.docx</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
@@ -1008,17 +1055,54 @@
       </c>
       <c r="E8" s="10" t="inlineStr">
         <is>
-          <t>Agente Etapa 3 (Analítica &amp; Gemini IA)</t>
+          <t>Servicio DUA Institucional</t>
         </is>
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>Generación del Informe Analítico Oficial con ficha muestral, estadística descriptiva/inferencial y prescripción multinivel.</t>
+          <t>Alineación curricular DUA (CAST 2024) para 12 estudiantes.</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
-          <t>Aseguramiento de la calidad académica según ISO 21001:2018 Cláusula 9.1.</t>
+          <t>Cumplimiento de equidad, inclusión educativa y principio de no discriminación (ISO 21001).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>EVT-005</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>06/09/2026 21:12</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Plan de Aprendizaje Modular CBL - FIS301 - Fisica Cuantica Aplicada</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>0.0 -&gt; 1.0</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>Motor de Planificación CBL / UbD</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>Compilación oficial del Plan de Aprendizaje Modular con alineamiento constructivo, créditos SCT e inclusión DUA.</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>Aseguramiento del diseño curricular modular bajo estándar ISO 21001:2018 Cláusula 7.5.</t>
         </is>
       </c>
     </row>

</xml_diff>